<commit_message>
Fix header merges: include col D in rows 3-9
</commit_message>
<xml_diff>
--- a/api/template.xlsx
+++ b/api/template.xlsx
@@ -326,7 +326,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -376,19 +376,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
@@ -402,37 +389,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -515,7 +472,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -527,7 +484,37 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
@@ -606,7 +593,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -619,134 +606,126 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="11" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1226,10 +1205,11 @@
         <v>3</v>
       </c>
       <c r="C3" s="5"/>
-      <c r="E3" s="6">
+      <c r="D3" s="6">
         <f>+TODAY()</f>
         <v>46192</v>
       </c>
+      <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -1246,18 +1226,19 @@
         <v>4</v>
       </c>
       <c r="C4" s="7"/>
-      <c r="E4" s="8" t="s">
+      <c r="D4" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
+      <c r="E4"/>
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
+      <c r="M4"/>
+      <c r="N4"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
@@ -1265,18 +1246,19 @@
         <v>6</v>
       </c>
       <c r="C5" s="7"/>
-      <c r="E5" s="8" t="s">
+      <c r="D5" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
+      <c r="E5"/>
+      <c r="F5"/>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+      <c r="M5"/>
+      <c r="N5"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
@@ -1284,18 +1266,19 @@
         <v>8</v>
       </c>
       <c r="C6" s="7"/>
-      <c r="E6" s="8" t="s">
+      <c r="D6" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
+      <c r="E6"/>
+      <c r="F6"/>
+      <c r="G6"/>
+      <c r="H6"/>
+      <c r="I6"/>
+      <c r="J6"/>
+      <c r="K6"/>
+      <c r="L6"/>
+      <c r="M6"/>
+      <c r="N6"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
@@ -1303,18 +1286,19 @@
         <v>10</v>
       </c>
       <c r="C7" s="7"/>
-      <c r="E7" s="8" t="s">
+      <c r="D7" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
+      <c r="E7"/>
+      <c r="F7"/>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7"/>
+      <c r="J7"/>
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7"/>
+      <c r="N7"/>
     </row>
     <row r="8" ht="15.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
@@ -1322,445 +1306,447 @@
         <v>12</v>
       </c>
       <c r="C8" s="7"/>
-      <c r="E8" s="8" t="s">
+      <c r="D8" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8"/>
+      <c r="N8"/>
     </row>
     <row r="9" ht="15.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="9"/>
-      <c r="E9" s="10" t="s">
+      <c r="C9" s="8"/>
+      <c r="D9" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9"/>
+      <c r="J9"/>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9"/>
+      <c r="N9"/>
     </row>
     <row r="10" ht="27" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="14" t="s">
+      <c r="F10" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="H10" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="I10" s="16" t="s">
+      <c r="I10" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="J10" s="14" t="s">
+      <c r="J10" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="K10" s="16" t="s">
+      <c r="K10" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="L10" s="14" t="s">
+      <c r="L10" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="M10" s="14" t="s">
+      <c r="M10" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="N10" s="17" t="s">
+      <c r="N10" s="15" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="14"/>
-      <c r="N11" s="17"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="15"/>
     </row>
     <row r="12" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="14"/>
-      <c r="N12" s="17"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="15"/>
     </row>
     <row r="13" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="18"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="26"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="27"/>
-      <c r="M13" s="27"/>
-      <c r="N13" s="28"/>
+      <c r="A13" s="16"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="25"/>
+      <c r="M13" s="25"/>
+      <c r="N13" s="26"/>
     </row>
     <row r="14" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="18"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="27"/>
-      <c r="M14" s="27"/>
-      <c r="N14" s="28"/>
+      <c r="A14" s="16"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="25"/>
+      <c r="M14" s="25"/>
+      <c r="N14" s="26"/>
     </row>
     <row r="15" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="18"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="26"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="27"/>
-      <c r="M15" s="27"/>
-      <c r="N15" s="28"/>
+      <c r="A15" s="16"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="25"/>
+      <c r="M15" s="25"/>
+      <c r="N15" s="26"/>
     </row>
     <row r="16" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="18"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="26"/>
-      <c r="K16" s="25"/>
-      <c r="L16" s="27"/>
-      <c r="M16" s="27"/>
-      <c r="N16" s="28"/>
+      <c r="A16" s="16"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="26"/>
     </row>
     <row r="17" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="18"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="26"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="27"/>
-      <c r="M17" s="27"/>
-      <c r="N17" s="28"/>
+      <c r="A17" s="16"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="26"/>
     </row>
     <row r="18" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="18"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="25"/>
-      <c r="L18" s="27"/>
-      <c r="M18" s="27"/>
-      <c r="N18" s="28"/>
+      <c r="A18" s="16"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="25"/>
+      <c r="M18" s="25"/>
+      <c r="N18" s="26"/>
     </row>
     <row r="19" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="18"/>
-      <c r="B19" s="19"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="25"/>
-      <c r="I19" s="25"/>
-      <c r="J19" s="26"/>
-      <c r="K19" s="25"/>
-      <c r="L19" s="27"/>
-      <c r="M19" s="27"/>
-      <c r="N19" s="28"/>
+      <c r="A19" s="16"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="24"/>
+      <c r="K19" s="23"/>
+      <c r="L19" s="25"/>
+      <c r="M19" s="25"/>
+      <c r="N19" s="26"/>
     </row>
     <row r="20" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="18"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="27"/>
-      <c r="M20" s="27"/>
-      <c r="N20" s="28"/>
+      <c r="A20" s="16"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="23"/>
+      <c r="L20" s="25"/>
+      <c r="M20" s="25"/>
+      <c r="N20" s="26"/>
     </row>
     <row r="21" ht="27.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="18"/>
-      <c r="B21" s="19"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="25"/>
-      <c r="L21" s="27"/>
-      <c r="M21" s="27"/>
-      <c r="N21" s="28"/>
+      <c r="A21" s="16"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="25"/>
+      <c r="M21" s="25"/>
+      <c r="N21" s="26"/>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="29"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="23"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="30"/>
-      <c r="J22" s="31"/>
-      <c r="K22" s="31"/>
-      <c r="L22" s="27"/>
-      <c r="M22" s="27"/>
-      <c r="N22" s="28"/>
+      <c r="A22" s="27"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="28"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
+      <c r="L22" s="25"/>
+      <c r="M22" s="25"/>
+      <c r="N22" s="26"/>
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="29"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="30"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="31"/>
-      <c r="L23" s="27"/>
-      <c r="M23" s="27"/>
-      <c r="N23" s="28"/>
+      <c r="A23" s="27"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="28"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="25"/>
+      <c r="M23" s="25"/>
+      <c r="N23" s="26"/>
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="32"/>
-      <c r="B24" s="33"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="35"/>
-      <c r="H24" s="35"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="37"/>
-      <c r="K24" s="35"/>
-      <c r="L24" s="35"/>
-      <c r="M24" s="38"/>
-      <c r="N24" s="39"/>
+      <c r="A24" s="30"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="34"/>
+      <c r="J24" s="35"/>
+      <c r="K24" s="33"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="36"/>
+      <c r="N24" s="37"/>
     </row>
     <row r="25" ht="22.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="40" t="s">
+      <c r="A25" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="40"/>
-      <c r="C25" s="40"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="40"/>
-      <c r="I25" s="41" t="s">
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="J25" s="41"/>
-      <c r="K25" s="42" t="s">
+      <c r="J25" s="39"/>
+      <c r="K25" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="L25" s="42"/>
-      <c r="M25" s="42"/>
-      <c r="N25" s="42"/>
+      <c r="L25" s="40"/>
+      <c r="M25" s="40"/>
+      <c r="N25" s="40"/>
     </row>
     <row r="26" ht="26.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="40"/>
-      <c r="B26" s="40"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="40"/>
-      <c r="F26" s="40"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="40"/>
-      <c r="I26" s="43" t="s">
+      <c r="A26" s="38"/>
+      <c r="B26" s="38"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="38"/>
+      <c r="I26" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="J26" s="44"/>
-      <c r="K26" s="42"/>
-      <c r="L26" s="42"/>
-      <c r="M26" s="42"/>
-      <c r="N26" s="42"/>
+      <c r="J26" s="42"/>
+      <c r="K26" s="40"/>
+      <c r="L26" s="40"/>
+      <c r="M26" s="40"/>
+      <c r="N26" s="40"/>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="40"/>
-      <c r="B27" s="40"/>
-      <c r="C27" s="40"/>
-      <c r="D27" s="40"/>
-      <c r="E27" s="40"/>
-      <c r="F27" s="40"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="43" t="s">
+      <c r="A27" s="38"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="J27" s="44"/>
-      <c r="K27" s="45"/>
-      <c r="L27" s="45"/>
-      <c r="M27" s="45"/>
-      <c r="N27" s="45"/>
+      <c r="J27" s="42"/>
+      <c r="K27" s="43"/>
+      <c r="L27" s="43"/>
+      <c r="M27" s="43"/>
+      <c r="N27" s="43"/>
     </row>
     <row r="28" ht="33" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="40"/>
-      <c r="B28" s="40"/>
-      <c r="C28" s="40"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="40"/>
-      <c r="I28" s="46" t="s">
+      <c r="A28" s="38"/>
+      <c r="B28" s="38"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="J28" s="47"/>
-      <c r="K28" s="45"/>
-      <c r="L28" s="45"/>
-      <c r="M28" s="45"/>
-      <c r="N28" s="45"/>
+      <c r="J28" s="45"/>
+      <c r="K28" s="43"/>
+      <c r="L28" s="43"/>
+      <c r="M28" s="43"/>
+      <c r="N28" s="43"/>
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="48" t="s">
+      <c r="A29" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="48"/>
-      <c r="G29" s="48"/>
-      <c r="H29" s="48"/>
-      <c r="I29" s="48"/>
-      <c r="J29" s="48"/>
-      <c r="K29" s="42" t="s">
+      <c r="B29" s="46"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="46"/>
+      <c r="I29" s="46"/>
+      <c r="J29" s="46"/>
+      <c r="K29" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="L29" s="42"/>
-      <c r="M29" s="42"/>
-      <c r="N29" s="42"/>
+      <c r="L29" s="40"/>
+      <c r="M29" s="40"/>
+      <c r="N29" s="40"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="48"/>
-      <c r="B30" s="48"/>
-      <c r="C30" s="48"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="48"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="48"/>
-      <c r="H30" s="48"/>
-      <c r="I30" s="48"/>
-      <c r="J30" s="48"/>
-      <c r="K30" s="49"/>
-      <c r="L30" s="49"/>
-      <c r="M30" s="49"/>
-      <c r="N30" s="49"/>
+      <c r="A30" s="46"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="46"/>
+      <c r="I30" s="46"/>
+      <c r="J30" s="46"/>
+      <c r="K30" s="47"/>
+      <c r="L30" s="47"/>
+      <c r="M30" s="47"/>
+      <c r="N30" s="47"/>
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="48"/>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="48"/>
-      <c r="H31" s="48"/>
-      <c r="I31" s="48"/>
-      <c r="J31" s="48"/>
-      <c r="K31" s="49"/>
-      <c r="L31" s="49"/>
-      <c r="M31" s="49"/>
-      <c r="N31" s="49"/>
-    </row>
-    <row r="32" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="E32" s="50"/>
-      <c r="F32" s="51"/>
-      <c r="G32" s="51"/>
-      <c r="H32" s="51"/>
-      <c r="I32" s="51"/>
-      <c r="J32" s="51"/>
-      <c r="K32" s="51"/>
-      <c r="L32" s="51"/>
-      <c r="M32" s="51"/>
-      <c r="N32" s="52"/>
+      <c r="A31" s="46"/>
+      <c r="B31" s="46"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="46"/>
+      <c r="I31" s="46"/>
+      <c r="J31" s="46"/>
+      <c r="K31" s="47"/>
+      <c r="L31" s="47"/>
+      <c r="M31" s="47"/>
+      <c r="N31" s="47"/>
+    </row>
+    <row r="32" spans="5:14" x14ac:dyDescent="0.25">
+      <c r="E32" s="48"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="49"/>
+      <c r="H32" s="49"/>
+      <c r="I32" s="49"/>
+      <c r="J32" s="49"/>
+      <c r="K32" s="49"/>
+      <c r="L32" s="49"/>
+      <c r="M32" s="49"/>
+      <c r="N32" s="50"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
@@ -1768,19 +1754,19 @@
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="A2:A9"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="E3:N3"/>
+    <mergeCell ref="D3:N3"/>
     <mergeCell ref="B4:C4"/>
-    <mergeCell ref="E4:N4"/>
+    <mergeCell ref="D4:N4"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="E5:N5"/>
+    <mergeCell ref="D5:N5"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="E6:N6"/>
+    <mergeCell ref="D6:N6"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="E7:N7"/>
+    <mergeCell ref="D7:N7"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="E8:N8"/>
+    <mergeCell ref="D8:N8"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="E9:N9"/>
+    <mergeCell ref="D9:N9"/>
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="C10:C12"/>

</xml_diff>